<commit_message>
fix tables headers in general.md
</commit_message>
<xml_diff>
--- a/SET_210.05-0/unit1.1.xlsx
+++ b/SET_210.05-0/unit1.1.xlsx
@@ -47,11 +47,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,80 +414,70 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Технические данные ИЧМ</t>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Параметр</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Значение</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Параметр</t>
+          <t>Код заказа ИЧМ</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Значение</t>
+          <t>ЮНИТ-ИЧМ-СУГР-С</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Код заказа ИЧМ</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>ЮНИТ-ИЧМ-СУГР-С</t>
-        </is>
-      </c>
+          <t>Заводской номер</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Заводской номер</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
+          <t>Завод-изготовитель</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ООО Юнител Инжиниринг</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Завод-изготовитель</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>ООО Юнител Инжиниринг</t>
-        </is>
-      </c>
+          <t>Год выпуска</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Год выпуска</t>
+          <t>Uпит, В</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Uпит, В</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>